<commit_message>
v1.3.2 — Réseau Air France refondu (sourcé indicateur 1956) + image d'accueil
- Air France : suppression des lignes reconstituées, remplacées par les 6 lignes
  Super Constellation relevées sur l'indicateur officiel Air France (été 1956) —
  « Parisien Spécial » (Paris–New York), prolongements Mexico (via NY / via Boston),
  Amérique du Sud (Paris–Buenos Aires via São Paulo/Montevideo), « Eastern Epicurean »
  (Paris–Tokyo via Téhéran/Manille), « L'Épicurien » (Paris–Londres). Vols retour [R].
- Image d'accueil (fond-accueil.jpg) affichée à sa taille d'origine quand aucune
  ligne n'est sélectionnée.
- Modale « À propos » : remerciement bilingue à Alexair (tables/images AF 1956).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/liaisons_Super_Constellation/Reseau_Air_France_L1049_sourced.xlsx
+++ b/liaisons_Super_Constellation/Reseau_Air_France_L1049_sourced.xlsx
@@ -4,7 +4,8 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Atlantique &amp; Amériques" sheetId="1" r:id="rId1"/>
-    <sheet name="Orient &amp; Afrique" sheetId="2" r:id="rId2"/>
+    <sheet name="Extrême-Orient" sheetId="2" r:id="rId2"/>
+    <sheet name="Europe" sheetId="3" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
@@ -398,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:L15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -423,190 +424,226 @@
         <v>Escale 3 (Arr. / Dép.)</v>
       </c>
       <c r="H1" t="str">
+        <v>Escale 4 (Arr. / Dép.)</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Escale 5 (Arr. / Dép.)</v>
+      </c>
+      <c r="J1" t="str">
         <v>Destination</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>Arrivée (HL)</v>
       </c>
-      <c r="J1" t="str">
+      <c r="L1" t="str">
         <v>Fréquence / Note</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>AF 017</v>
+        <v>AF 045</v>
       </c>
       <c r="B2" t="str">
-        <v>Atlantique Nord (Le Parisien)</v>
+        <v>Atlantique Nord (Parisien Spécial)</v>
       </c>
       <c r="C2" t="str">
         <v>Paris (ORY)</v>
       </c>
       <c r="D2" t="str">
-        <v>20:00</v>
+        <v>23:00</v>
       </c>
       <c r="E2" t="str">
-        <v>Shannon (22:45 / 23:45)</v>
+        <v>-</v>
       </c>
       <c r="F2" t="str">
-        <v>Gander [Tech] (05:30 / 06:45 *)</v>
+        <v>-</v>
       </c>
       <c r="G2" t="str">
         <v>-</v>
       </c>
       <c r="H2" t="str">
+        <v>-</v>
+      </c>
+      <c r="I2" t="str">
+        <v>-</v>
+      </c>
+      <c r="J2" t="str">
         <v>New York (IDL)</v>
       </c>
-      <c r="I2" t="str">
-        <v>10:15 *</v>
-      </c>
-      <c r="J2" t="str">
-        <v>Ligne prestige (nuit)</v>
+      <c r="K2" t="str">
+        <v>08:40 *</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Quotidien</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>AF 018</v>
+        <v>AF 046</v>
       </c>
       <c r="B3" t="str">
-        <v>Atlantique Nord (Retour)</v>
+        <v>Atlantique Nord (Parisien Spécial) (Retour)</v>
       </c>
       <c r="C3" t="str">
         <v>New York (IDL)</v>
       </c>
       <c r="D3" t="str">
-        <v>16:30</v>
+        <v>19:00</v>
       </c>
       <c r="E3" t="str">
-        <v>Gander [Tech] (21:45 / 22:45)</v>
+        <v>-</v>
       </c>
       <c r="F3" t="str">
-        <v>Shannon (07:30 / 08:30 *)</v>
+        <v>-</v>
       </c>
       <c r="G3" t="str">
         <v>-</v>
       </c>
       <c r="H3" t="str">
+        <v>-</v>
+      </c>
+      <c r="I3" t="str">
+        <v>-</v>
+      </c>
+      <c r="J3" t="str">
         <v>Paris (ORY)</v>
       </c>
-      <c r="I3" t="str">
-        <v>11:45 *</v>
-      </c>
-      <c r="J3" t="str">
-        <v>Vol de nuit</v>
+      <c r="K3" t="str">
+        <v>08:00 *</v>
+      </c>
+      <c r="L3" t="str">
+        <v>Quotidien</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>AF 211</v>
+        <v>AF 079</v>
       </c>
       <c r="B4" t="str">
-        <v>Antilles &amp; Amérique Centrale</v>
+        <v>Atlantique Nord (Mexico via Boston)</v>
       </c>
       <c r="C4" t="str">
         <v>Paris (ORY)</v>
       </c>
       <c r="D4" t="str">
-        <v>10:00</v>
+        <v>22:00</v>
       </c>
       <c r="E4" t="str">
-        <v>Santa Maria (15:00 / 16:15)</v>
+        <v>Boston (BOS) (08:40 * / 09:20 *)</v>
       </c>
       <c r="F4" t="str">
-        <v>Pointe-à-Pitre (00:30 / 02:00 *)</v>
+        <v>New York (IDL) (10:30 * / 12:00 *)</v>
       </c>
       <c r="G4" t="str">
-        <v>Caracas (05:00 / 06:15 *)</v>
+        <v>-</v>
       </c>
       <c r="H4" t="str">
-        <v>Bogota (BOG)</v>
+        <v>-</v>
       </c>
       <c r="I4" t="str">
-        <v>08:15 *</v>
+        <v>-</v>
       </c>
       <c r="J4" t="str">
-        <v>Route des Antilles</v>
+        <v>Mexico (MEX)</v>
+      </c>
+      <c r="K4" t="str">
+        <v>17:55 *</v>
+      </c>
+      <c r="L4" t="str">
+        <v>Mardi, Jeudi, Samedi</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>AF 212</v>
+        <v>AF 080</v>
       </c>
       <c r="B5" t="str">
-        <v>Antilles &amp; Amérique Centrale (Retour)</v>
+        <v>Atlantique Nord (Mexico via Boston) (Retour)</v>
       </c>
       <c r="C5" t="str">
-        <v>Bogota (BOG)</v>
+        <v>Mexico (MEX)</v>
       </c>
       <c r="D5" t="str">
-        <v>16:00</v>
+        <v>08:00</v>
       </c>
       <c r="E5" t="str">
-        <v>Caracas (18:00 / 19:15)</v>
+        <v>New York (IDL) (13:35 / 15:00)</v>
       </c>
       <c r="F5" t="str">
-        <v>Pointe-à-Pitre (22:15 / 23:45)</v>
+        <v>Boston (BOS) (16:00 / 17:00)</v>
       </c>
       <c r="G5" t="str">
-        <v>Santa Maria (08:00 * / 09:15 *)</v>
+        <v>-</v>
       </c>
       <c r="H5" t="str">
+        <v>-</v>
+      </c>
+      <c r="I5" t="str">
+        <v>-</v>
+      </c>
+      <c r="J5" t="str">
         <v>Paris (ORY)</v>
       </c>
-      <c r="I5" t="str">
-        <v>14:15 *</v>
-      </c>
-      <c r="J5" t="str">
-        <v>Route des Antilles</v>
+      <c r="K5" t="str">
+        <v>06:30 *</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Mercredi, Vendredi, Dimanche</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>AF 501</v>
+        <v>AF 071</v>
       </c>
       <c r="B6" t="str">
-        <v>Atlantique Sud</v>
+        <v>Atlantique Nord (Mexico)</v>
       </c>
       <c r="C6" t="str">
         <v>Paris (ORY)</v>
       </c>
       <c r="D6" t="str">
-        <v>18:30</v>
+        <v>22:00</v>
       </c>
       <c r="E6" t="str">
-        <v>Casablanca (22:15 / 23:30)</v>
+        <v>New York (IDL) (09:20 * / 12:00 *)</v>
       </c>
       <c r="F6" t="str">
-        <v>Dakar (06:00 / 07:30 *)</v>
+        <v>-</v>
       </c>
       <c r="G6" t="str">
-        <v>Recife (16:00 / 17:00 *)</v>
+        <v>-</v>
       </c>
       <c r="H6" t="str">
-        <v>Rio de Janeiro (GIG)</v>
+        <v>-</v>
       </c>
       <c r="I6" t="str">
-        <v>21:30 *</v>
+        <v>-</v>
       </c>
       <c r="J6" t="str">
-        <v>Prolongé Buenos Aires</v>
+        <v>Mexico (MEX)</v>
+      </c>
+      <c r="K6" t="str">
+        <v>17:55 *</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Quotidien</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>AF 502</v>
+        <v>AF 072</v>
       </c>
       <c r="B7" t="str">
-        <v>Atlantique Sud (Tronçon final)</v>
+        <v>Atlantique Nord (Mexico) (Retour)</v>
       </c>
       <c r="C7" t="str">
-        <v>Rio de Janeiro (GIG)</v>
+        <v>Mexico (MEX)</v>
       </c>
       <c r="D7" t="str">
-        <v>08:00</v>
+        <v>09:00</v>
       </c>
       <c r="E7" t="str">
-        <v>-</v>
+        <v>New York (IDL) (14:35 / 16:30)</v>
       </c>
       <c r="F7" t="str">
         <v>-</v>
@@ -615,77 +652,95 @@
         <v>-</v>
       </c>
       <c r="H7" t="str">
-        <v>Buenos Aires (EZE)</v>
+        <v>-</v>
       </c>
       <c r="I7" t="str">
-        <v>11:30</v>
+        <v>-</v>
       </c>
       <c r="J7" t="str">
-        <v>Correspondance AF 501</v>
+        <v>Paris (ORY)</v>
+      </c>
+      <c r="K7" t="str">
+        <v>06:00 *</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Quotidien</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>AF 503</v>
+        <v>AF 093</v>
       </c>
       <c r="B8" t="str">
-        <v>Atlantique Sud (Retour)</v>
+        <v>Amérique du Sud</v>
       </c>
       <c r="C8" t="str">
+        <v>Paris (ORY)</v>
+      </c>
+      <c r="D8" t="str">
+        <v>13:00</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Madrid (15:45 / 16:45)</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Dakar (23:20 / 00:35 *)</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Rio de Janeiro (GIG) (09:00 * / 10:15 *)</v>
+      </c>
+      <c r="H8" t="str">
+        <v>São Paulo (CGH) (11:40 * / 12:25 *)</v>
+      </c>
+      <c r="I8" t="str">
+        <v>Montevideo (16:25 * / 16:55 *)</v>
+      </c>
+      <c r="J8" t="str">
         <v>Buenos Aires (EZE)</v>
       </c>
-      <c r="D8" t="str">
-        <v>08:00</v>
-      </c>
-      <c r="E8" t="str">
-        <v>-</v>
-      </c>
-      <c r="F8" t="str">
-        <v>-</v>
-      </c>
-      <c r="G8" t="str">
-        <v>-</v>
-      </c>
-      <c r="H8" t="str">
-        <v>Rio de Janeiro (GIG)</v>
-      </c>
-      <c r="I8" t="str">
-        <v>11:30</v>
-      </c>
-      <c r="J8" t="str">
-        <v>Tronçon initial (corr. AF 504)</v>
+      <c r="K8" t="str">
+        <v>17:50 *</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Jeudi, Dimanche</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>AF 504</v>
+        <v>AF 094</v>
       </c>
       <c r="B9" t="str">
-        <v>Atlantique Sud (Retour)</v>
+        <v>Amérique du Sud (Retour)</v>
       </c>
       <c r="C9" t="str">
-        <v>Rio de Janeiro (GIG)</v>
+        <v>Buenos Aires (EZE)</v>
       </c>
       <c r="D9" t="str">
-        <v>13:00</v>
+        <v>09:00</v>
       </c>
       <c r="E9" t="str">
-        <v>Recife (17:30 / 18:30)</v>
+        <v>Montevideo (09:55 / 10:25)</v>
       </c>
       <c r="F9" t="str">
-        <v>Dakar (DKR) (03:00 * / 04:30 *)</v>
+        <v>São Paulo (CGH) (14:00 / 14:45)</v>
       </c>
       <c r="G9" t="str">
-        <v>Casablanca (11:00 * / 12:15 *)</v>
+        <v>Rio de Janeiro (GIG) (16:00 / 17:00)</v>
       </c>
       <c r="H9" t="str">
+        <v>Dakar (01:30 * / 02:45 *)</v>
+      </c>
+      <c r="I9" t="str">
+        <v>Madrid (11:30 * / 12:30 *)</v>
+      </c>
+      <c r="J9" t="str">
         <v>Paris (ORY)</v>
       </c>
-      <c r="I9" t="str">
-        <v>16:00 *</v>
-      </c>
-      <c r="J9" t="str">
-        <v>Depuis Buenos Aires (corr. AF 503)</v>
+      <c r="K9" t="str">
+        <v>14:45 *</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Lundi, Vendredi</v>
       </c>
     </row>
     <row r="10">
@@ -717,6 +772,12 @@
         <v/>
       </c>
       <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
+        <v/>
+      </c>
+      <c r="L10" t="str">
         <v/>
       </c>
     </row>
@@ -751,6 +812,12 @@
       <c r="J11" t="str">
         <v/>
       </c>
+      <c r="K11" t="str">
+        <v/>
+      </c>
+      <c r="L11" t="str">
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -783,10 +850,16 @@
       <c r="J12" t="str">
         <v/>
       </c>
+      <c r="K12" t="str">
+        <v/>
+      </c>
+      <c r="L12" t="str">
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>[S] Sourcé : axes réellement ouverts au L-1049C dès 1953 — Paris–New York, Paris–Buenos Aires, Pointe-à-Pitre, Caracas, Tokyo ; escales techniques Gander/Shannon.</v>
+        <v>[S] Sourcé : réseau et horaires d'après l'indicateur officiel Air France (été 1956) — « Parisien Spécial » (Paris–New York), prolongements vers Mexico (via New York ou via Boston) et Amérique du Sud (AF 093) Paris–Madrid–Dakar–Rio–São Paulo–Montevideo–Buenos Aires.</v>
       </c>
       <c r="B13" t="str">
         <v/>
@@ -813,12 +886,18 @@
         <v/>
       </c>
       <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
+        <v/>
+      </c>
+      <c r="L13" t="str">
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>[R] Reconstitué : numéros de vol et horaires — plausibles mais non issus d'un timetable original.</v>
+        <v>[R] Vols retour reconstitués (itinéraire miroir) : horaires ALLER conformes à l'indicateur Air France 1956, horaires RETOUR plausibles.</v>
       </c>
       <c r="B14" t="str">
         <v/>
@@ -845,6 +924,12 @@
         <v/>
       </c>
       <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
+        <v/>
+      </c>
+      <c r="L14" t="str">
         <v/>
       </c>
     </row>
@@ -879,81 +964,23 @@
       <c r="J15" t="str">
         <v/>
       </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>[R] Vols retour ajoutés automatiquement (itinéraire miroir, horaires reconstitués).</v>
-      </c>
-      <c r="B16" t="str">
-        <v/>
-      </c>
-      <c r="C16" t="str">
-        <v/>
-      </c>
-      <c r="D16" t="str">
-        <v/>
-      </c>
-      <c r="E16" t="str">
-        <v/>
-      </c>
-      <c r="F16" t="str">
-        <v/>
-      </c>
-      <c r="G16" t="str">
-        <v/>
-      </c>
-      <c r="H16" t="str">
-        <v/>
-      </c>
-      <c r="I16" t="str">
-        <v/>
-      </c>
-      <c r="J16" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>[R] AF 503/504 : service inverse complet de l’Atlantique Sud (Buenos Aires → Rio → Recife → Dakar → Casablanca → Paris), reconstitué.</v>
-      </c>
-      <c r="B17" t="str">
-        <v/>
-      </c>
-      <c r="C17" t="str">
-        <v/>
-      </c>
-      <c r="D17" t="str">
-        <v/>
-      </c>
-      <c r="E17" t="str">
-        <v/>
-      </c>
-      <c r="F17" t="str">
-        <v/>
-      </c>
-      <c r="G17" t="str">
-        <v/>
-      </c>
-      <c r="H17" t="str">
-        <v/>
-      </c>
-      <c r="I17" t="str">
-        <v/>
-      </c>
-      <c r="J17" t="str">
+      <c r="K15" t="str">
+        <v/>
+      </c>
+      <c r="L15" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L15"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:M8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -984,59 +1011,65 @@
         <v>Escale 5 (Arr. / Dép.)</v>
       </c>
       <c r="J1" t="str">
+        <v>Escale 6 (Arr. / Dép.)</v>
+      </c>
+      <c r="K1" t="str">
         <v>Destination</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Arrivée (HL)</v>
       </c>
-      <c r="L1" t="str">
-        <v>Note</v>
+      <c r="M1" t="str">
+        <v>Fréquence / Note</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>AF 184</v>
+        <v>AF 170</v>
       </c>
       <c r="B2" t="str">
-        <v>Extrême-Orient (Le Tokyo)</v>
+        <v>Extrême-Orient (Eastern Epicurean)</v>
       </c>
       <c r="C2" t="str">
         <v>Paris (ORY)</v>
       </c>
       <c r="D2" t="str">
-        <v>13:00 (Mer)</v>
+        <v>17:40</v>
       </c>
       <c r="E2" t="str">
-        <v>Rome (17:00 / 18:00)</v>
+        <v>Rome (20:30 / 21:50)</v>
       </c>
       <c r="F2" t="str">
-        <v>Beyrouth (23:30 / 00:45 *)</v>
+        <v>Téhéran (08:30 * / 10:00 *)</v>
       </c>
       <c r="G2" t="str">
-        <v>Karachi (08:30 / 09:45 *)</v>
+        <v>Karachi (16:00 * / 17:30 *)</v>
       </c>
       <c r="H2" t="str">
-        <v>Calcutta (15:00 / 16:15 *)</v>
+        <v>Bangkok (03:50 ** / 04:50 **)</v>
       </c>
       <c r="I2" t="str">
-        <v>Saïgon (23:30 * / 01:00)</v>
+        <v>Saïgon (06:40 ** / 08:10 **)</v>
       </c>
       <c r="J2" t="str">
+        <v>Manille (13:10 ** / 14:10 **)</v>
+      </c>
+      <c r="K2" t="str">
         <v>Tokyo (HND)</v>
       </c>
-      <c r="K2" t="str">
-        <v>15:30 (Ven)</v>
-      </c>
       <c r="L2" t="str">
-        <v>Ligne du Cap au Japon</v>
+        <v>22:15 **</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Mardi, Samedi</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>AF 185</v>
+        <v>AF 171</v>
       </c>
       <c r="B3" t="str">
-        <v>Extrême-Orient (Le Tokyo) (Retour)</v>
+        <v>Extrême-Orient (Eastern Epicurean) (Retour)</v>
       </c>
       <c r="C3" t="str">
         <v>Tokyo (HND)</v>
@@ -1045,185 +1078,200 @@
         <v>16:00</v>
       </c>
       <c r="E3" t="str">
-        <v>Saïgon (06:30 * / 08:00 *)</v>
+        <v>Manille (20:00 / 21:00)</v>
       </c>
       <c r="F3" t="str">
-        <v>Calcutta (15:15 * / 16:30 *)</v>
+        <v>Saïgon (01:15 * / 02:15 *)</v>
       </c>
       <c r="G3" t="str">
-        <v>Karachi (21:45 * / 23:00 *)</v>
+        <v>Bangkok (04:00 * / 05:00 *)</v>
       </c>
       <c r="H3" t="str">
-        <v>Beyrouth (06:45 ** / 08:00 **)</v>
+        <v>Karachi (12:00 * / 13:00 *)</v>
       </c>
       <c r="I3" t="str">
-        <v>Rome (13:30 ** / 14:30 **)</v>
+        <v>Téhéran (18:00 * / 19:00 *)</v>
       </c>
       <c r="J3" t="str">
+        <v>Rome (01:30 ** / 02:30 **)</v>
+      </c>
+      <c r="K3" t="str">
         <v>Paris (ORY)</v>
       </c>
-      <c r="K3" t="str">
-        <v>18:30 **</v>
-      </c>
       <c r="L3" t="str">
-        <v>Ligne du Cap au Japon</v>
+        <v>05:30 **</v>
+      </c>
+      <c r="M3" t="str">
+        <v>Jeudi, Dimanche</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>AF 186</v>
+        <v/>
       </c>
       <c r="B4" t="str">
-        <v>Indochine (Saïgon)</v>
+        <v/>
       </c>
       <c r="C4" t="str">
-        <v>Paris (ORY)</v>
+        <v/>
       </c>
       <c r="D4" t="str">
-        <v>14:00 (Mer)</v>
+        <v/>
       </c>
       <c r="E4" t="str">
-        <v>Rome (18:00 / 19:00)</v>
+        <v/>
       </c>
       <c r="F4" t="str">
-        <v>Le Caire (CAI) (23:30 / 00:45 *)</v>
+        <v/>
       </c>
       <c r="G4" t="str">
-        <v>Karachi (08:00 / 09:15 *)</v>
+        <v/>
       </c>
       <c r="H4" t="str">
-        <v>Calcutta (14:30 / 15:45 *)</v>
+        <v/>
       </c>
       <c r="I4" t="str">
-        <v>Bangkok (BKK) (21:00 / 22:15 *)</v>
+        <v/>
       </c>
       <c r="J4" t="str">
-        <v>Saïgon (SGN)</v>
+        <v/>
       </c>
       <c r="K4" t="str">
-        <v>01:30 (Ven)</v>
+        <v/>
       </c>
       <c r="L4" t="str">
-        <v>Courrier d’Indochine</v>
+        <v/>
+      </c>
+      <c r="M4" t="str">
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>AF 187</v>
+        <v>Notes :</v>
       </c>
       <c r="B5" t="str">
-        <v>Indochine (Saïgon) (Retour)</v>
+        <v/>
       </c>
       <c r="C5" t="str">
-        <v>Saïgon (SGN)</v>
+        <v/>
       </c>
       <c r="D5" t="str">
-        <v>16:00</v>
+        <v/>
       </c>
       <c r="E5" t="str">
-        <v>Bangkok (BKK) (19:15 / 20:30)</v>
+        <v/>
       </c>
       <c r="F5" t="str">
-        <v>Calcutta (01:45 * / 03:00 *)</v>
+        <v/>
       </c>
       <c r="G5" t="str">
-        <v>Karachi (08:15 * / 09:30 *)</v>
+        <v/>
       </c>
       <c r="H5" t="str">
-        <v>Le Caire (CAI) (16:45 * / 18:00 *)</v>
+        <v/>
       </c>
       <c r="I5" t="str">
-        <v>Rome (22:30 * / 23:30 *)</v>
+        <v/>
       </c>
       <c r="J5" t="str">
-        <v>Paris (ORY)</v>
+        <v/>
       </c>
       <c r="K5" t="str">
-        <v>03:30 **</v>
+        <v/>
       </c>
       <c r="L5" t="str">
-        <v>Courrier d’Indochine</v>
+        <v/>
+      </c>
+      <c r="M5" t="str">
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>AF 405</v>
+        <v>[S] Sourcé : le service « Eastern Epicurean » (AF 170, Super Constellation) reliait Paris–Rome–Téhéran–Karachi–Bangkok–Saïgon–Manille–Tokyo, d'après l'indicateur officiel Air France (été 1956).</v>
       </c>
       <c r="B6" t="str">
-        <v>Afrique Centrale</v>
+        <v/>
       </c>
       <c r="C6" t="str">
-        <v>Paris (ORY)</v>
+        <v/>
       </c>
       <c r="D6" t="str">
-        <v>22:30</v>
+        <v/>
       </c>
       <c r="E6" t="str">
-        <v>Alger (01:45 / 02:45 *)</v>
+        <v/>
       </c>
       <c r="F6" t="str">
-        <v>Kano [Tech] (10:15 / 11:30 *)</v>
+        <v/>
       </c>
       <c r="G6" t="str">
-        <v>-</v>
+        <v/>
       </c>
       <c r="H6" t="str">
-        <v>-</v>
+        <v/>
       </c>
       <c r="I6" t="str">
-        <v>-</v>
+        <v/>
       </c>
       <c r="J6" t="str">
-        <v>Brazzaville (BZV)</v>
+        <v/>
       </c>
       <c r="K6" t="str">
-        <v>16:45 *</v>
+        <v/>
       </c>
       <c r="L6" t="str">
-        <v>Axe transsaharien</v>
+        <v/>
+      </c>
+      <c r="M6" t="str">
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>AF 406</v>
+        <v>[R] Vol retour reconstitué (itinéraire miroir) ; horaires aller conformes à l'indicateur, retour plausible.</v>
       </c>
       <c r="B7" t="str">
-        <v>Afrique Centrale (Retour)</v>
+        <v/>
       </c>
       <c r="C7" t="str">
-        <v>Brazzaville (BZV)</v>
+        <v/>
       </c>
       <c r="D7" t="str">
-        <v>16:00</v>
+        <v/>
       </c>
       <c r="E7" t="str">
-        <v>Kano [Tech] (21:15 / 22:30)</v>
+        <v/>
       </c>
       <c r="F7" t="str">
-        <v>Alger (06:00 * / 07:00 *)</v>
+        <v/>
       </c>
       <c r="G7" t="str">
-        <v>-</v>
+        <v/>
       </c>
       <c r="H7" t="str">
-        <v>-</v>
+        <v/>
       </c>
       <c r="I7" t="str">
-        <v>-</v>
+        <v/>
       </c>
       <c r="J7" t="str">
-        <v>Paris (ORY)</v>
+        <v/>
       </c>
       <c r="K7" t="str">
-        <v>10:15 *</v>
+        <v/>
       </c>
       <c r="L7" t="str">
-        <v>Axe transsaharien</v>
+        <v/>
+      </c>
+      <c r="M7" t="str">
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v/>
+        <v>* / ** : arrivée à J+1 / J+2. HL : Heure Locale.</v>
       </c>
       <c r="B8" t="str">
         <v/>
@@ -1258,200 +1306,208 @@
       <c r="L8" t="str">
         <v/>
       </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>Notes :</v>
-      </c>
-      <c r="B9" t="str">
-        <v/>
-      </c>
-      <c r="C9" t="str">
-        <v/>
-      </c>
-      <c r="D9" t="str">
-        <v/>
-      </c>
-      <c r="E9" t="str">
-        <v/>
-      </c>
-      <c r="F9" t="str">
-        <v/>
-      </c>
-      <c r="G9" t="str">
-        <v/>
-      </c>
-      <c r="H9" t="str">
-        <v/>
-      </c>
-      <c r="I9" t="str">
-        <v/>
-      </c>
-      <c r="J9" t="str">
-        <v/>
-      </c>
-      <c r="K9" t="str">
-        <v/>
-      </c>
-      <c r="L9" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>[S] Sourcé : Air France exploite le L-1049 vers l'Extrême-Orient (Tokyo, Saïgon/Indochine) et l'Afrique centrale ; corridors et escales conformes à l'époque.</v>
-      </c>
-      <c r="B10" t="str">
-        <v/>
-      </c>
-      <c r="C10" t="str">
-        <v/>
-      </c>
-      <c r="D10" t="str">
-        <v/>
-      </c>
-      <c r="E10" t="str">
-        <v/>
-      </c>
-      <c r="F10" t="str">
-        <v/>
-      </c>
-      <c r="G10" t="str">
-        <v/>
-      </c>
-      <c r="H10" t="str">
-        <v/>
-      </c>
-      <c r="I10" t="str">
-        <v/>
-      </c>
-      <c r="J10" t="str">
-        <v/>
-      </c>
-      <c r="K10" t="str">
-        <v/>
-      </c>
-      <c r="L10" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>[R] Reconstitué : numéros de vol et horaires exacts.</v>
-      </c>
-      <c r="B11" t="str">
-        <v/>
-      </c>
-      <c r="C11" t="str">
-        <v/>
-      </c>
-      <c r="D11" t="str">
-        <v/>
-      </c>
-      <c r="E11" t="str">
-        <v/>
-      </c>
-      <c r="F11" t="str">
-        <v/>
-      </c>
-      <c r="G11" t="str">
-        <v/>
-      </c>
-      <c r="H11" t="str">
-        <v/>
-      </c>
-      <c r="I11" t="str">
-        <v/>
-      </c>
-      <c r="J11" t="str">
-        <v/>
-      </c>
-      <c r="K11" t="str">
-        <v/>
-      </c>
-      <c r="L11" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>* Arrivée le lendemain (+1 jour). (Mer)/(Ven) = jour de circulation. [Tech] = escale technique.</v>
-      </c>
-      <c r="B12" t="str">
-        <v/>
-      </c>
-      <c r="C12" t="str">
-        <v/>
-      </c>
-      <c r="D12" t="str">
-        <v/>
-      </c>
-      <c r="E12" t="str">
-        <v/>
-      </c>
-      <c r="F12" t="str">
-        <v/>
-      </c>
-      <c r="G12" t="str">
-        <v/>
-      </c>
-      <c r="H12" t="str">
-        <v/>
-      </c>
-      <c r="I12" t="str">
-        <v/>
-      </c>
-      <c r="J12" t="str">
-        <v/>
-      </c>
-      <c r="K12" t="str">
-        <v/>
-      </c>
-      <c r="L12" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>[R] Vols retour ajoutés automatiquement (itinéraire miroir, horaires reconstitués).</v>
-      </c>
-      <c r="B13" t="str">
-        <v/>
-      </c>
-      <c r="C13" t="str">
-        <v/>
-      </c>
-      <c r="D13" t="str">
-        <v/>
-      </c>
-      <c r="E13" t="str">
-        <v/>
-      </c>
-      <c r="F13" t="str">
-        <v/>
-      </c>
-      <c r="G13" t="str">
-        <v/>
-      </c>
-      <c r="H13" t="str">
-        <v/>
-      </c>
-      <c r="I13" t="str">
-        <v/>
-      </c>
-      <c r="J13" t="str">
-        <v/>
-      </c>
-      <c r="K13" t="str">
-        <v/>
-      </c>
-      <c r="L13" t="str">
+      <c r="M8" t="str">
         <v/>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M8"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G8"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>N° Vol</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Axe / Ligne</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Origine</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Départ (HL)</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Destination</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Arrivée (HL)</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Fréquence / Note</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>AF 568</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Europe (Épicurien)</v>
+      </c>
+      <c r="C2" t="str">
+        <v>Paris (ORY)</v>
+      </c>
+      <c r="D2" t="str">
+        <v>12:00</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Londres (LHR)</v>
+      </c>
+      <c r="F2" t="str">
+        <v>13:15</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Quotidien</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>AF 569</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Europe (Épicurien) (Retour)</v>
+      </c>
+      <c r="C3" t="str">
+        <v>Londres (LHR)</v>
+      </c>
+      <c r="D3" t="str">
+        <v>14:00</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Paris (ORY)</v>
+      </c>
+      <c r="F3" t="str">
+        <v>15:15</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Quotidien</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v/>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Notes :</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>[S] Sourcé : le service « L'Épicurien » (AF 568, Super Constellation) reliait Paris (Orly, 12:00) à Londres (13:15), d'après l'indicateur officiel Air France (été 1956) ; vol court de prestige.</v>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v/>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+      <c r="F6" t="str">
+        <v/>
+      </c>
+      <c r="G6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>[R] Vol retour reconstitué (Londres–Paris) ; horaire aller conforme à l'indicateur Air France 1956.</v>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v/>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v/>
+      </c>
+      <c r="G7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>HL : Heure Locale.</v>
+      </c>
+      <c r="B8" t="str">
+        <v/>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v/>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v/>
+      </c>
+      <c r="G8" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:G8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>